<commit_message>
Scale demo to realistic starter revenue
</commit_message>
<xml_diff>
--- a/examples/dana-automates-business-demo.xlsx
+++ b/examples/dana-automates-business-demo.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R0b7a97afd9c340b6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Invoices" sheetId="2" r:id="Rc0d879097d304ae7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Customers" sheetId="3" r:id="Rb8c0f675d06b4ba7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sales" sheetId="4" r:id="Rd0554be6e88544ab"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" r:id="R64b14077f54c4081"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Invoices" sheetId="2" r:id="R28d975d977e748de"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Customers" sheetId="3" r:id="R874cac960e584f46"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sales" sheetId="4" r:id="Rae67f95d3bb7440f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -174,7 +174,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="57">
+  <x:cellXfs count="59">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -188,7 +188,9 @@
     <x:xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="200" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="201" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="201" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -556,7 +558,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R530558fdd13c4ab6"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R9fa5b7b4d6694b7e"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -586,7 +588,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="Rb12ee43d9e404f4f"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R1e1a04c4ecce4c99"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -596,7 +598,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="InvoicesTable" displayName="InvoicesTable" ref="A4:H16" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="InvoicesTable" displayName="InvoicesTable" ref="A4:H12" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="8">
     <x:tableColumn id="1" name="Invoice"/>
     <x:tableColumn id="2" name="Client"/>
@@ -612,7 +614,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="CustomersTable" displayName="CustomersTable" ref="A4:J19" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="CustomersTable" displayName="CustomersTable" ref="A4:J12" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="10">
     <x:tableColumn id="1" name="Customer ID"/>
     <x:tableColumn id="2" name="Business"/>
@@ -630,7 +632,7 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="SalesTable" displayName="SalesTable" ref="A4:F22" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="SalesTable" displayName="SalesTable" ref="A4:F14" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
   <x:tableColumns count="6">
     <x:tableColumn id="1" name="Date"/>
     <x:tableColumn id="2" name="Client"/>
@@ -853,190 +855,190 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="36" customHeight="1">
-      <x:c r="A1" s="10" t="str">
+      <x:c r="A1" s="12" t="str">
         <x:v>DANA AUTOMATES • BUSINESS DASHBOARD</x:v>
       </x:c>
-      <x:c r="B1" s="10"/>
-      <x:c r="C1" s="10"/>
-      <x:c r="D1" s="10"/>
-      <x:c r="E1" s="10"/>
-      <x:c r="F1" s="10"/>
-      <x:c r="G1" s="10"/>
-      <x:c r="H1" s="10"/>
-      <x:c r="I1" s="10"/>
-      <x:c r="J1" s="10"/>
-      <x:c r="K1" s="10"/>
-      <x:c r="L1" s="10"/>
+      <x:c r="B1" s="12"/>
+      <x:c r="C1" s="12"/>
+      <x:c r="D1" s="12"/>
+      <x:c r="E1" s="12"/>
+      <x:c r="F1" s="12"/>
+      <x:c r="G1" s="12"/>
+      <x:c r="H1" s="12"/>
+      <x:c r="I1" s="12"/>
+      <x:c r="J1" s="12"/>
+      <x:c r="K1" s="12"/>
+      <x:c r="L1" s="12"/>
     </x:row>
     <x:row r="2">
-      <x:c r="A2" s="11" t="str">
+      <x:c r="A2" s="13" t="str">
         <x:v>Live formulas linked to the invoice, customer and sales sheets</x:v>
       </x:c>
-      <x:c r="B2" s="11"/>
-      <x:c r="C2" s="11"/>
-      <x:c r="D2" s="11"/>
-      <x:c r="E2" s="11"/>
-      <x:c r="F2" s="11"/>
-      <x:c r="G2" s="11"/>
-      <x:c r="H2" s="11"/>
-      <x:c r="I2" s="11"/>
-      <x:c r="J2" s="11"/>
-      <x:c r="K2" s="11"/>
-      <x:c r="L2" s="11"/>
+      <x:c r="B2" s="13"/>
+      <x:c r="C2" s="13"/>
+      <x:c r="D2" s="13"/>
+      <x:c r="E2" s="13"/>
+      <x:c r="F2" s="13"/>
+      <x:c r="G2" s="13"/>
+      <x:c r="H2" s="13"/>
+      <x:c r="I2" s="13"/>
+      <x:c r="J2" s="13"/>
+      <x:c r="K2" s="13"/>
+      <x:c r="L2" s="13"/>
     </x:row>
     <x:row r="4">
-      <x:c r="A4" s="14" t="str">
+      <x:c r="A4" s="16" t="str">
         <x:v>Total revenue</x:v>
       </x:c>
-      <x:c r="B4" s="14"/>
-      <x:c r="C4" s="14"/>
-      <x:c r="E4" s="37" t="str">
+      <x:c r="B4" s="16"/>
+      <x:c r="C4" s="16"/>
+      <x:c r="E4" s="39" t="str">
         <x:v>Outstanding invoices</x:v>
       </x:c>
-      <x:c r="F4" s="37"/>
-      <x:c r="G4" s="37"/>
-      <x:c r="I4" s="40" t="str">
+      <x:c r="F4" s="39"/>
+      <x:c r="G4" s="39"/>
+      <x:c r="I4" s="42" t="str">
         <x:v>Active customers</x:v>
       </x:c>
-      <x:c r="J4" s="40"/>
-      <x:c r="K4" s="40"/>
+      <x:c r="J4" s="42"/>
+      <x:c r="K4" s="42"/>
     </x:row>
     <x:row r="5">
-      <x:c r="A5" s="41" t="n">
+      <x:c r="A5" s="43" t="n">
         <x:f>SUM('Sales'!D5:D22)</x:f>
-        <x:v>37100</x:v>
-      </x:c>
-      <x:c r="B5" s="42"/>
-      <x:c r="C5" s="43"/>
-      <x:c r="E5" s="41" t="n">
+        <x:v>10800</x:v>
+      </x:c>
+      <x:c r="B5" s="44"/>
+      <x:c r="C5" s="45"/>
+      <x:c r="E5" s="43" t="n">
         <x:f>SUMIF('Invoices'!G5:G16,"&lt;&gt;Paid",'Invoices'!F5:F16)</x:f>
-        <x:v>23950</x:v>
-      </x:c>
-      <x:c r="F5" s="42"/>
-      <x:c r="G5" s="43"/>
-      <x:c r="I5" s="47" t="n">
+        <x:v>6900</x:v>
+      </x:c>
+      <x:c r="F5" s="44"/>
+      <x:c r="G5" s="45"/>
+      <x:c r="I5" s="49" t="n">
         <x:f>COUNTIF('Customers'!H5:H19,"Active")</x:f>
-        <x:v>10</x:v>
-      </x:c>
-      <x:c r="J5" s="48"/>
-      <x:c r="K5" s="49"/>
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="J5" s="50"/>
+      <x:c r="K5" s="51"/>
     </x:row>
     <x:row r="6">
-      <x:c r="A6" s="44"/>
-      <x:c r="B6" s="45"/>
-      <x:c r="C6" s="46"/>
-      <x:c r="E6" s="44"/>
-      <x:c r="F6" s="45"/>
-      <x:c r="G6" s="46"/>
-      <x:c r="I6" s="50"/>
-      <x:c r="J6" s="51"/>
-      <x:c r="K6" s="52"/>
+      <x:c r="A6" s="46"/>
+      <x:c r="B6" s="47"/>
+      <x:c r="C6" s="48"/>
+      <x:c r="E6" s="46"/>
+      <x:c r="F6" s="47"/>
+      <x:c r="G6" s="48"/>
+      <x:c r="I6" s="52"/>
+      <x:c r="J6" s="53"/>
+      <x:c r="K6" s="54"/>
     </x:row>
     <x:row r="9">
-      <x:c r="A9" s="55" t="str">
+      <x:c r="A9" s="57" t="str">
         <x:v>Status</x:v>
       </x:c>
-      <x:c r="B9" s="55" t="str">
+      <x:c r="B9" s="57" t="str">
         <x:v>Count</x:v>
       </x:c>
-      <x:c r="C9" s="53"/>
-      <x:c r="D9" s="55" t="str">
+      <x:c r="C9" s="55"/>
+      <x:c r="D9" s="57" t="str">
         <x:v>Service</x:v>
       </x:c>
-      <x:c r="E9" s="55" t="str">
+      <x:c r="E9" s="57" t="str">
         <x:v>Revenue</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
-      <x:c r="A10" s="53" t="str">
+      <x:c r="A10" s="55" t="str">
         <x:v>Draft</x:v>
       </x:c>
-      <x:c r="B10" s="53" t="n">
+      <x:c r="B10" s="55" t="n">
         <x:f>COUNTIF('Invoices'!G5:G16,A10)</x:f>
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="C10" s="53"/>
-      <x:c r="D10" s="53" t="str">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C10" s="55"/>
+      <x:c r="D10" s="55" t="str">
         <x:v>Admin Automation</x:v>
       </x:c>
-      <x:c r="E10" s="56" t="n">
+      <x:c r="E10" s="58" t="n">
         <x:f>SUMIF('Sales'!C5:C22,D10,'Sales'!D5:D22)</x:f>
-        <x:v>5850</x:v>
+        <x:v>900</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
-      <x:c r="A11" s="53" t="str">
+      <x:c r="A11" s="55" t="str">
         <x:v>Sent</x:v>
       </x:c>
-      <x:c r="B11" s="53" t="n">
+      <x:c r="B11" s="55" t="n">
         <x:f>COUNTIF('Invoices'!G5:G16,A11)</x:f>
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="C11" s="53"/>
-      <x:c r="D11" s="53" t="str">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C11" s="55"/>
+      <x:c r="D11" s="55" t="str">
         <x:v>Reporting</x:v>
       </x:c>
-      <x:c r="E11" s="56" t="n">
+      <x:c r="E11" s="58" t="n">
         <x:f>SUMIF('Sales'!C5:C22,D11,'Sales'!D5:D22)</x:f>
-        <x:v>8000</x:v>
+        <x:v>3200</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
-      <x:c r="A12" s="53" t="str">
+      <x:c r="A12" s="55" t="str">
         <x:v>Paid</x:v>
       </x:c>
-      <x:c r="B12" s="53" t="n">
+      <x:c r="B12" s="55" t="n">
         <x:f>COUNTIF('Invoices'!G5:G16,A12)</x:f>
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="C12" s="53"/>
-      <x:c r="D12" s="53" t="str">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="C12" s="55"/>
+      <x:c r="D12" s="55" t="str">
         <x:v>Follow-ups</x:v>
       </x:c>
-      <x:c r="E12" s="56" t="n">
+      <x:c r="E12" s="58" t="n">
         <x:f>SUMIF('Sales'!C5:C22,D12,'Sales'!D5:D22)</x:f>
-        <x:v>6700</x:v>
+        <x:v>3100</x:v>
       </x:c>
     </x:row>
     <x:row r="13">
-      <x:c r="A13" s="53" t="str">
+      <x:c r="A13" s="55" t="str">
         <x:v>Overdue</x:v>
       </x:c>
-      <x:c r="B13" s="53" t="n">
+      <x:c r="B13" s="55" t="n">
         <x:f>COUNTIF('Invoices'!G5:G16,A13)</x:f>
         <x:v>2</x:v>
       </x:c>
-      <x:c r="C13" s="53"/>
-      <x:c r="D13" s="53" t="str">
+      <x:c r="C13" s="55"/>
+      <x:c r="D13" s="55" t="str">
         <x:v>Data Filing</x:v>
       </x:c>
-      <x:c r="E13" s="56" t="n">
+      <x:c r="E13" s="58" t="n">
         <x:f>SUMIF('Sales'!C5:C22,D13,'Sales'!D5:D22)</x:f>
-        <x:v>6050</x:v>
+        <x:v>1800</x:v>
       </x:c>
     </x:row>
     <x:row r="14">
-      <x:c r="A14" s="53"/>
-      <x:c r="B14" s="53"/>
-      <x:c r="C14" s="53"/>
-      <x:c r="D14" s="53" t="str">
+      <x:c r="A14" s="55"/>
+      <x:c r="B14" s="55"/>
+      <x:c r="C14" s="55"/>
+      <x:c r="D14" s="55" t="str">
         <x:v>Dashboard</x:v>
       </x:c>
-      <x:c r="E14" s="56" t="n">
+      <x:c r="E14" s="58" t="n">
         <x:f>SUMIF('Sales'!C5:C22,D14,'Sales'!D5:D22)</x:f>
-        <x:v>4800</x:v>
+        <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
-      <x:c r="A15" s="53"/>
-      <x:c r="B15" s="53"/>
-      <x:c r="C15" s="53"/>
-      <x:c r="D15" s="53" t="str">
+      <x:c r="A15" s="55"/>
+      <x:c r="B15" s="55"/>
+      <x:c r="C15" s="55"/>
+      <x:c r="D15" s="55" t="str">
         <x:v>Other</x:v>
       </x:c>
-      <x:c r="E15" s="56" t="n">
+      <x:c r="E15" s="58" t="n">
         <x:f>SUM('Sales'!D5:D22)-SUM(E10:E14)</x:f>
-        <x:v>5700</x:v>
+        <x:v>1800</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1051,7 +1053,7 @@
     <x:mergeCell ref="I5:K6"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7514920703994578"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd5389ec8e6324d67"/>
 </x:worksheet>
 </file>
 
@@ -1145,8 +1147,8 @@
       <x:c r="E5" s="8" t="n">
         <x:v>46199</x:v>
       </x:c>
-      <x:c r="F5" s="9" t="n">
-        <x:v>4250</x:v>
+      <x:c r="F5" s="10" t="n">
+        <x:v>1200</x:v>
       </x:c>
       <x:c r="G5" s="7" t="str">
         <x:v>Overdue</x:v>
@@ -1171,8 +1173,8 @@
       <x:c r="E6" s="8" t="n">
         <x:v>46205</x:v>
       </x:c>
-      <x:c r="F6" s="9" t="n">
-        <x:v>1850</x:v>
+      <x:c r="F6" s="10" t="n">
+        <x:v>900</x:v>
       </x:c>
       <x:c r="G6" s="7" t="str">
         <x:v>Overdue</x:v>
@@ -1197,8 +1199,8 @@
       <x:c r="E7" s="8" t="n">
         <x:v>46209</x:v>
       </x:c>
-      <x:c r="F7" s="9" t="n">
-        <x:v>3200</x:v>
+      <x:c r="F7" s="10" t="n">
+        <x:v>1800</x:v>
       </x:c>
       <x:c r="G7" s="7" t="str">
         <x:v>Sent</x:v>
@@ -1223,8 +1225,8 @@
       <x:c r="E8" s="8" t="n">
         <x:v>46212</x:v>
       </x:c>
-      <x:c r="F8" s="9" t="n">
-        <x:v>950</x:v>
+      <x:c r="F8" s="10" t="n">
+        <x:v>750</x:v>
       </x:c>
       <x:c r="G8" s="7" t="str">
         <x:v>Sent</x:v>
@@ -1249,8 +1251,8 @@
       <x:c r="E9" s="8" t="n">
         <x:v>46214</x:v>
       </x:c>
-      <x:c r="F9" s="9" t="n">
-        <x:v>2100</x:v>
+      <x:c r="F9" s="10" t="n">
+        <x:v>1100</x:v>
       </x:c>
       <x:c r="G9" s="7" t="str">
         <x:v>Paid</x:v>
@@ -1275,8 +1277,8 @@
       <x:c r="E10" s="8" t="n">
         <x:v>46215</x:v>
       </x:c>
-      <x:c r="F10" s="9" t="n">
-        <x:v>2750</x:v>
+      <x:c r="F10" s="10" t="n">
+        <x:v>600</x:v>
       </x:c>
       <x:c r="G10" s="7" t="str">
         <x:v>Paid</x:v>
@@ -1301,8 +1303,8 @@
       <x:c r="E11" s="8" t="n">
         <x:v>46218</x:v>
       </x:c>
-      <x:c r="F11" s="9" t="n">
-        <x:v>1450</x:v>
+      <x:c r="F11" s="10" t="n">
+        <x:v>850</x:v>
       </x:c>
       <x:c r="G11" s="7" t="str">
         <x:v>Draft</x:v>
@@ -1327,8 +1329,8 @@
       <x:c r="E12" s="8" t="n">
         <x:v>46219</x:v>
       </x:c>
-      <x:c r="F12" s="9" t="n">
-        <x:v>3600</x:v>
+      <x:c r="F12" s="10" t="n">
+        <x:v>1400</x:v>
       </x:c>
       <x:c r="G12" s="7" t="str">
         <x:v>Draft</x:v>
@@ -1338,108 +1340,24 @@
       </x:c>
     </x:row>
     <x:row r="13">
-      <x:c r="A13" s="7" t="str">
-        <x:v>INV-2026-049</x:v>
-      </x:c>
-      <x:c r="B13" s="7" t="str">
-        <x:v>Khayelitsha Kitchens</x:v>
-      </x:c>
-      <x:c r="C13" s="7" t="str">
-        <x:v>orders@kkitchens.example</x:v>
-      </x:c>
-      <x:c r="D13" s="8" t="n">
-        <x:v>46206</x:v>
-      </x:c>
-      <x:c r="E13" s="8" t="n">
-        <x:v>46220</x:v>
-      </x:c>
-      <x:c r="F13" s="9" t="n">
-        <x:v>1250</x:v>
-      </x:c>
-      <x:c r="G13" s="7" t="str">
-        <x:v>Paid</x:v>
-      </x:c>
-      <x:c r="H13" s="7" t="str">
-        <x:v>Order filing workflow</x:v>
-      </x:c>
+      <x:c r="D13" s="9"/>
+      <x:c r="E13" s="9"/>
+      <x:c r="F13" s="11"/>
     </x:row>
     <x:row r="14">
-      <x:c r="A14" s="7" t="str">
-        <x:v>INV-2026-050</x:v>
-      </x:c>
-      <x:c r="B14" s="7" t="str">
-        <x:v>Pretoria Pet Care</x:v>
-      </x:c>
-      <x:c r="C14" s="7" t="str">
-        <x:v>care@pretoriapets.example</x:v>
-      </x:c>
-      <x:c r="D14" s="8" t="n">
-        <x:v>46207</x:v>
-      </x:c>
-      <x:c r="E14" s="8" t="n">
-        <x:v>46221</x:v>
-      </x:c>
-      <x:c r="F14" s="9" t="n">
-        <x:v>2200</x:v>
-      </x:c>
-      <x:c r="G14" s="7" t="str">
-        <x:v>Sent</x:v>
-      </x:c>
-      <x:c r="H14" s="7" t="str">
-        <x:v>Appointment reminders</x:v>
-      </x:c>
+      <x:c r="D14" s="9"/>
+      <x:c r="E14" s="9"/>
+      <x:c r="F14" s="11"/>
     </x:row>
     <x:row r="15">
-      <x:c r="A15" s="7" t="str">
-        <x:v>INV-2026-051</x:v>
-      </x:c>
-      <x:c r="B15" s="7" t="str">
-        <x:v>Vuka Consulting</x:v>
-      </x:c>
-      <x:c r="C15" s="7" t="str">
-        <x:v>team@vukaconsulting.example</x:v>
-      </x:c>
-      <x:c r="D15" s="8" t="n">
-        <x:v>46208</x:v>
-      </x:c>
-      <x:c r="E15" s="8" t="n">
-        <x:v>46222</x:v>
-      </x:c>
-      <x:c r="F15" s="9" t="n">
-        <x:v>4800</x:v>
-      </x:c>
-      <x:c r="G15" s="7" t="str">
-        <x:v>Draft</x:v>
-      </x:c>
-      <x:c r="H15" s="7" t="str">
-        <x:v>Client reporting dashboard</x:v>
-      </x:c>
+      <x:c r="D15" s="9"/>
+      <x:c r="E15" s="9"/>
+      <x:c r="F15" s="11"/>
     </x:row>
     <x:row r="16">
-      <x:c r="A16" s="7" t="str">
-        <x:v>INV-2026-052</x:v>
-      </x:c>
-      <x:c r="B16" s="7" t="str">
-        <x:v>Durban Design Co</x:v>
-      </x:c>
-      <x:c r="C16" s="7" t="str">
-        <x:v>studio@durbandesign.example</x:v>
-      </x:c>
-      <x:c r="D16" s="8" t="n">
-        <x:v>46209</x:v>
-      </x:c>
-      <x:c r="E16" s="8" t="n">
-        <x:v>46223</x:v>
-      </x:c>
-      <x:c r="F16" s="9" t="n">
-        <x:v>1650</x:v>
-      </x:c>
-      <x:c r="G16" s="7" t="str">
-        <x:v>Sent</x:v>
-      </x:c>
-      <x:c r="H16" s="7" t="str">
-        <x:v>Asset filing automation</x:v>
-      </x:c>
+      <x:c r="D16" s="9"/>
+      <x:c r="E16" s="9"/>
+      <x:c r="F16" s="11"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -1457,7 +1375,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Reda0e70b03cc4a23"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5449cb8b4c7742fc"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1807,228 +1725,25 @@
       </x:c>
     </x:row>
     <x:row r="13">
-      <x:c r="A13" s="7" t="str">
-        <x:v>C-009</x:v>
-      </x:c>
-      <x:c r="B13" s="7" t="str">
-        <x:v>Khayelitsha Kitchens</x:v>
-      </x:c>
-      <x:c r="C13" s="7" t="str">
-        <x:v>Zanele Mayekiso</x:v>
-      </x:c>
-      <x:c r="D13" s="7" t="str">
-        <x:v>zanele@kkitchens.example</x:v>
-      </x:c>
-      <x:c r="E13" s="7" t="str">
-        <x:v>071 560 8044</x:v>
-      </x:c>
-      <x:c r="F13" s="7" t="str">
-        <x:v>Cape Town</x:v>
-      </x:c>
-      <x:c r="G13" s="7" t="str">
-        <x:v>Food</x:v>
-      </x:c>
-      <x:c r="H13" s="7" t="str">
-        <x:v>Active</x:v>
-      </x:c>
-      <x:c r="I13" s="8" t="n">
-        <x:v>46166</x:v>
-      </x:c>
-      <x:c r="J13" s="7" t="str">
-        <x:v>Order exports arrive daily</x:v>
-      </x:c>
+      <x:c r="I13" s="9"/>
     </x:row>
     <x:row r="14">
-      <x:c r="A14" s="7" t="str">
-        <x:v>C-010</x:v>
-      </x:c>
-      <x:c r="B14" s="7" t="str">
-        <x:v>Pretoria Pet Care</x:v>
-      </x:c>
-      <x:c r="C14" s="7" t="str">
-        <x:v>Anika van Wyk</x:v>
-      </x:c>
-      <x:c r="D14" s="7" t="str">
-        <x:v>anika@pretoriapets.example</x:v>
-      </x:c>
-      <x:c r="E14" s="7" t="str">
-        <x:v>084 310 9952</x:v>
-      </x:c>
-      <x:c r="F14" s="7" t="str">
-        <x:v>Pretoria</x:v>
-      </x:c>
-      <x:c r="G14" s="7" t="str">
-        <x:v>Pet Care</x:v>
-      </x:c>
-      <x:c r="H14" s="7" t="str">
-        <x:v>Lead</x:v>
-      </x:c>
-      <x:c r="I14" s="8" t="n">
-        <x:v>46174</x:v>
-      </x:c>
-      <x:c r="J14" s="7" t="str">
-        <x:v>Wants WhatsApp pricing first</x:v>
-      </x:c>
+      <x:c r="I14" s="9"/>
     </x:row>
     <x:row r="15">
-      <x:c r="A15" s="7" t="str">
-        <x:v>C-011</x:v>
-      </x:c>
-      <x:c r="B15" s="7" t="str">
-        <x:v>Vuka Consulting</x:v>
-      </x:c>
-      <x:c r="C15" s="7" t="str">
-        <x:v>Refilwe Seopa</x:v>
-      </x:c>
-      <x:c r="D15" s="7" t="str">
-        <x:v>refilwe@vukaconsulting.example</x:v>
-      </x:c>
-      <x:c r="E15" s="7" t="str">
-        <x:v>082 441 8720</x:v>
-      </x:c>
-      <x:c r="F15" s="7" t="str">
-        <x:v>Sandton</x:v>
-      </x:c>
-      <x:c r="G15" s="7" t="str">
-        <x:v>Consulting</x:v>
-      </x:c>
-      <x:c r="H15" s="7" t="str">
-        <x:v>Active</x:v>
-      </x:c>
-      <x:c r="I15" s="8" t="n">
-        <x:v>46182</x:v>
-      </x:c>
-      <x:c r="J15" s="7" t="str">
-        <x:v>Executive dashboard prospect</x:v>
-      </x:c>
+      <x:c r="I15" s="9"/>
     </x:row>
     <x:row r="16">
-      <x:c r="A16" s="7" t="str">
-        <x:v>C-012</x:v>
-      </x:c>
-      <x:c r="B16" s="7" t="str">
-        <x:v>Durban Design Co</x:v>
-      </x:c>
-      <x:c r="C16" s="7" t="str">
-        <x:v>Priya Naidoo</x:v>
-      </x:c>
-      <x:c r="D16" s="7" t="str">
-        <x:v>priya@durbandesign.example</x:v>
-      </x:c>
-      <x:c r="E16" s="7" t="str">
-        <x:v>074 905 1163</x:v>
-      </x:c>
-      <x:c r="F16" s="7" t="str">
-        <x:v>Durban</x:v>
-      </x:c>
-      <x:c r="G16" s="7" t="str">
-        <x:v>Creative</x:v>
-      </x:c>
-      <x:c r="H16" s="7" t="str">
-        <x:v>Active</x:v>
-      </x:c>
-      <x:c r="I16" s="8" t="n">
-        <x:v>46189</x:v>
-      </x:c>
-      <x:c r="J16" s="7" t="str">
-        <x:v>Shared-drive cleanup</x:v>
-      </x:c>
+      <x:c r="I16" s="9"/>
     </x:row>
     <x:row r="17">
-      <x:c r="A17" s="7" t="str">
-        <x:v>C-013</x:v>
-      </x:c>
-      <x:c r="B17" s="7" t="str">
-        <x:v>Soweto Solar</x:v>
-      </x:c>
-      <x:c r="C17" s="7" t="str">
-        <x:v>Neo Tshabalala</x:v>
-      </x:c>
-      <x:c r="D17" s="7" t="str">
-        <x:v>neo@sowetosolar.example</x:v>
-      </x:c>
-      <x:c r="E17" s="7" t="str">
-        <x:v>083 670 4512</x:v>
-      </x:c>
-      <x:c r="F17" s="7" t="str">
-        <x:v>Soweto</x:v>
-      </x:c>
-      <x:c r="G17" s="7" t="str">
-        <x:v>Energy</x:v>
-      </x:c>
-      <x:c r="H17" s="7" t="str">
-        <x:v>Lead</x:v>
-      </x:c>
-      <x:c r="I17" s="8" t="n">
-        <x:v>46198</x:v>
-      </x:c>
-      <x:c r="J17" s="7" t="str">
-        <x:v>Site inspection scheduling</x:v>
-      </x:c>
+      <x:c r="I17" s="9"/>
     </x:row>
     <x:row r="18">
-      <x:c r="A18" s="7" t="str">
-        <x:v>C-014</x:v>
-      </x:c>
-      <x:c r="B18" s="7" t="str">
-        <x:v>Garden Route Dental</x:v>
-      </x:c>
-      <x:c r="C18" s="7" t="str">
-        <x:v>Dr Emma Smith</x:v>
-      </x:c>
-      <x:c r="D18" s="7" t="str">
-        <x:v>emma@gardendental.example</x:v>
-      </x:c>
-      <x:c r="E18" s="7" t="str">
-        <x:v>072 334 8501</x:v>
-      </x:c>
-      <x:c r="F18" s="7" t="str">
-        <x:v>George</x:v>
-      </x:c>
-      <x:c r="G18" s="7" t="str">
-        <x:v>Healthcare</x:v>
-      </x:c>
-      <x:c r="H18" s="7" t="str">
-        <x:v>Inactive</x:v>
-      </x:c>
-      <x:c r="I18" s="8" t="n">
-        <x:v>46061</x:v>
-      </x:c>
-      <x:c r="J18" s="7" t="str">
-        <x:v>Paused project until Q4</x:v>
-      </x:c>
+      <x:c r="I18" s="9"/>
     </x:row>
     <x:row r="19">
-      <x:c r="A19" s="7" t="str">
-        <x:v>C-015</x:v>
-      </x:c>
-      <x:c r="B19" s="7" t="str">
-        <x:v>Bloem Bookkeeping</x:v>
-      </x:c>
-      <x:c r="C19" s="7" t="str">
-        <x:v>Karabo Mokoena</x:v>
-      </x:c>
-      <x:c r="D19" s="7" t="str">
-        <x:v>karabo@bloembooks.example</x:v>
-      </x:c>
-      <x:c r="E19" s="7" t="str">
-        <x:v>079 222 1376</x:v>
-      </x:c>
-      <x:c r="F19" s="7" t="str">
-        <x:v>Bloemfontein</x:v>
-      </x:c>
-      <x:c r="G19" s="7" t="str">
-        <x:v>Finance</x:v>
-      </x:c>
-      <x:c r="H19" s="7" t="str">
-        <x:v>Active</x:v>
-      </x:c>
-      <x:c r="I19" s="8" t="n">
-        <x:v>46203</x:v>
-      </x:c>
-      <x:c r="J19" s="7" t="str">
-        <x:v>Recurring month-end exports</x:v>
-      </x:c>
+      <x:c r="I19" s="9"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -2046,7 +1761,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R422f7a2c0f864d2e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3e9cdb9178c54b84"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -2129,8 +1844,8 @@
       <x:c r="C5" s="7" t="str">
         <x:v>Reporting</x:v>
       </x:c>
-      <x:c r="D5" s="9" t="n">
-        <x:v>3200</x:v>
+      <x:c r="D5" s="10" t="n">
+        <x:v>1200</x:v>
       </x:c>
       <x:c r="E5" s="7" t="str">
         <x:v>New</x:v>
@@ -2151,8 +1866,8 @@
       <x:c r="C6" s="7" t="str">
         <x:v>Admin Automation</x:v>
       </x:c>
-      <x:c r="D6" s="9" t="n">
-        <x:v>1850</x:v>
+      <x:c r="D6" s="10" t="n">
+        <x:v>900</x:v>
       </x:c>
       <x:c r="E6" s="7" t="str">
         <x:v>New</x:v>
@@ -2173,8 +1888,8 @@
       <x:c r="C7" s="7" t="str">
         <x:v>Website</x:v>
       </x:c>
-      <x:c r="D7" s="9" t="n">
-        <x:v>4250</x:v>
+      <x:c r="D7" s="10" t="n">
+        <x:v>1800</x:v>
       </x:c>
       <x:c r="E7" s="7" t="str">
         <x:v>New</x:v>
@@ -2195,8 +1910,8 @@
       <x:c r="C8" s="7" t="str">
         <x:v>Follow-ups</x:v>
       </x:c>
-      <x:c r="D8" s="9" t="n">
-        <x:v>2100</x:v>
+      <x:c r="D8" s="10" t="n">
+        <x:v>750</x:v>
       </x:c>
       <x:c r="E8" s="7" t="str">
         <x:v>New</x:v>
@@ -2217,8 +1932,8 @@
       <x:c r="C9" s="7" t="str">
         <x:v>Follow-ups</x:v>
       </x:c>
-      <x:c r="D9" s="9" t="n">
-        <x:v>2750</x:v>
+      <x:c r="D9" s="10" t="n">
+        <x:v>1100</x:v>
       </x:c>
       <x:c r="E9" s="7" t="str">
         <x:v>New</x:v>
@@ -2239,8 +1954,8 @@
       <x:c r="C10" s="7" t="str">
         <x:v>Reporting</x:v>
       </x:c>
-      <x:c r="D10" s="9" t="n">
-        <x:v>1200</x:v>
+      <x:c r="D10" s="10" t="n">
+        <x:v>600</x:v>
       </x:c>
       <x:c r="E10" s="7" t="str">
         <x:v>Recurring</x:v>
@@ -2261,8 +1976,8 @@
       <x:c r="C11" s="7" t="str">
         <x:v>Data Filing</x:v>
       </x:c>
-      <x:c r="D11" s="9" t="n">
-        <x:v>1250</x:v>
+      <x:c r="D11" s="10" t="n">
+        <x:v>850</x:v>
       </x:c>
       <x:c r="E11" s="7" t="str">
         <x:v>New</x:v>
@@ -2283,8 +1998,8 @@
       <x:c r="C12" s="7" t="str">
         <x:v>Reporting</x:v>
       </x:c>
-      <x:c r="D12" s="9" t="n">
-        <x:v>3600</x:v>
+      <x:c r="D12" s="10" t="n">
+        <x:v>1400</x:v>
       </x:c>
       <x:c r="E12" s="7" t="str">
         <x:v>New</x:v>
@@ -2305,8 +2020,8 @@
       <x:c r="C13" s="7" t="str">
         <x:v>Data Filing</x:v>
       </x:c>
-      <x:c r="D13" s="9" t="n">
-        <x:v>1650</x:v>
+      <x:c r="D13" s="10" t="n">
+        <x:v>950</x:v>
       </x:c>
       <x:c r="E13" s="7" t="str">
         <x:v>New</x:v>
@@ -2327,8 +2042,8 @@
       <x:c r="C14" s="7" t="str">
         <x:v>Follow-ups</x:v>
       </x:c>
-      <x:c r="D14" s="9" t="n">
-        <x:v>900</x:v>
+      <x:c r="D14" s="10" t="n">
+        <x:v>1250</x:v>
       </x:c>
       <x:c r="E14" s="7" t="str">
         <x:v>Recurring</x:v>
@@ -2340,180 +2055,36 @@
       <x:c r="H14" s="7"/>
     </x:row>
     <x:row r="15">
-      <x:c r="A15" s="8" t="n">
-        <x:v>46193</x:v>
-      </x:c>
-      <x:c r="B15" s="7" t="str">
-        <x:v>Mokoena Repairs</x:v>
-      </x:c>
-      <x:c r="C15" s="7" t="str">
-        <x:v>Admin Automation</x:v>
-      </x:c>
-      <x:c r="D15" s="9" t="n">
-        <x:v>1100</x:v>
-      </x:c>
-      <x:c r="E15" s="7" t="str">
-        <x:v>Recurring</x:v>
-      </x:c>
-      <x:c r="F15" s="7" t="str">
-        <x:v>Direct</x:v>
-      </x:c>
-      <x:c r="G15" s="7"/>
-      <x:c r="H15" s="7"/>
+      <x:c r="A15" s="9"/>
+      <x:c r="D15" s="11"/>
     </x:row>
     <x:row r="16">
-      <x:c r="A16" s="8" t="n">
-        <x:v>46200</x:v>
-      </x:c>
-      <x:c r="B16" s="7" t="str">
-        <x:v>Bloem Bookkeeping</x:v>
-      </x:c>
-      <x:c r="C16" s="7" t="str">
-        <x:v>Data Filing</x:v>
-      </x:c>
-      <x:c r="D16" s="9" t="n">
-        <x:v>2300</x:v>
-      </x:c>
-      <x:c r="E16" s="7" t="str">
-        <x:v>New</x:v>
-      </x:c>
-      <x:c r="F16" s="7" t="str">
-        <x:v>Referral</x:v>
-      </x:c>
-      <x:c r="G16" s="7"/>
-      <x:c r="H16" s="7"/>
+      <x:c r="A16" s="9"/>
+      <x:c r="D16" s="11"/>
     </x:row>
     <x:row r="17">
-      <x:c r="A17" s="8" t="n">
-        <x:v>46204</x:v>
-      </x:c>
-      <x:c r="B17" s="7" t="str">
-        <x:v>Pretoria Pet Care</x:v>
-      </x:c>
-      <x:c r="C17" s="7" t="str">
-        <x:v>Admin Automation</x:v>
-      </x:c>
-      <x:c r="D17" s="9" t="n">
-        <x:v>2200</x:v>
-      </x:c>
-      <x:c r="E17" s="7" t="str">
-        <x:v>New</x:v>
-      </x:c>
-      <x:c r="F17" s="7" t="str">
-        <x:v>Google</x:v>
-      </x:c>
-      <x:c r="G17" s="7"/>
-      <x:c r="H17" s="7"/>
+      <x:c r="A17" s="9"/>
+      <x:c r="D17" s="11"/>
     </x:row>
     <x:row r="18">
-      <x:c r="A18" s="8" t="n">
-        <x:v>46205</x:v>
-      </x:c>
-      <x:c r="B18" s="7" t="str">
-        <x:v>Jozi Auto Care</x:v>
-      </x:c>
-      <x:c r="C18" s="7" t="str">
-        <x:v>Follow-ups</x:v>
-      </x:c>
-      <x:c r="D18" s="9" t="n">
-        <x:v>950</x:v>
-      </x:c>
-      <x:c r="E18" s="7" t="str">
-        <x:v>Recurring</x:v>
-      </x:c>
-      <x:c r="F18" s="7" t="str">
-        <x:v>Direct</x:v>
-      </x:c>
-      <x:c r="G18" s="7"/>
-      <x:c r="H18" s="7"/>
+      <x:c r="A18" s="9"/>
+      <x:c r="D18" s="11"/>
     </x:row>
     <x:row r="19">
-      <x:c r="A19" s="8" t="n">
-        <x:v>46206</x:v>
-      </x:c>
-      <x:c r="B19" s="7" t="str">
-        <x:v>Vuka Consulting</x:v>
-      </x:c>
-      <x:c r="C19" s="7" t="str">
-        <x:v>Dashboard</x:v>
-      </x:c>
-      <x:c r="D19" s="9" t="n">
-        <x:v>4800</x:v>
-      </x:c>
-      <x:c r="E19" s="7" t="str">
-        <x:v>New</x:v>
-      </x:c>
-      <x:c r="F19" s="7" t="str">
-        <x:v>LinkedIn</x:v>
-      </x:c>
-      <x:c r="G19" s="7"/>
-      <x:c r="H19" s="7"/>
+      <x:c r="A19" s="9"/>
+      <x:c r="D19" s="11"/>
     </x:row>
     <x:row r="20">
-      <x:c r="A20" s="8" t="n">
-        <x:v>46207</x:v>
-      </x:c>
-      <x:c r="B20" s="7" t="str">
-        <x:v>Northside Hair Studio</x:v>
-      </x:c>
-      <x:c r="C20" s="7" t="str">
-        <x:v>Admin Automation</x:v>
-      </x:c>
-      <x:c r="D20" s="9" t="n">
-        <x:v>700</x:v>
-      </x:c>
-      <x:c r="E20" s="7" t="str">
-        <x:v>Recurring</x:v>
-      </x:c>
-      <x:c r="F20" s="7" t="str">
-        <x:v>Direct</x:v>
-      </x:c>
-      <x:c r="G20" s="7"/>
-      <x:c r="H20" s="7"/>
+      <x:c r="A20" s="9"/>
+      <x:c r="D20" s="11"/>
     </x:row>
     <x:row r="21">
-      <x:c r="A21" s="8" t="n">
-        <x:v>46208</x:v>
-      </x:c>
-      <x:c r="B21" s="7" t="str">
-        <x:v>Khayelitsha Kitchens</x:v>
-      </x:c>
-      <x:c r="C21" s="7" t="str">
-        <x:v>Data Filing</x:v>
-      </x:c>
-      <x:c r="D21" s="9" t="n">
-        <x:v>850</x:v>
-      </x:c>
-      <x:c r="E21" s="7" t="str">
-        <x:v>Recurring</x:v>
-      </x:c>
-      <x:c r="F21" s="7" t="str">
-        <x:v>Direct</x:v>
-      </x:c>
-      <x:c r="G21" s="7"/>
-      <x:c r="H21" s="7"/>
+      <x:c r="A21" s="9"/>
+      <x:c r="D21" s="11"/>
     </x:row>
     <x:row r="22">
-      <x:c r="A22" s="8" t="n">
-        <x:v>46209</x:v>
-      </x:c>
-      <x:c r="B22" s="7" t="str">
-        <x:v>Lerato Events</x:v>
-      </x:c>
-      <x:c r="C22" s="7" t="str">
-        <x:v>Spreadsheet Cleanup</x:v>
-      </x:c>
-      <x:c r="D22" s="9" t="n">
-        <x:v>1450</x:v>
-      </x:c>
-      <x:c r="E22" s="7" t="str">
-        <x:v>New</x:v>
-      </x:c>
-      <x:c r="F22" s="7" t="str">
-        <x:v>Instagram</x:v>
-      </x:c>
-      <x:c r="G22" s="7"/>
-      <x:c r="H22" s="7"/>
+      <x:c r="A22" s="9"/>
+      <x:c r="D22" s="11"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -2522,7 +2093,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf1b056b2a8984bcc"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9377dbfa9a11442e"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>